<commit_message>
Updated social registry fields and import template
</commit_message>
<xml_diff>
--- a/custom_import_template/static/xls/individual_import_template.xlsx
+++ b/custom_import_template/static/xls/individual_import_template.xlsx
@@ -544,13 +544,7 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="3">
-    <dataValidation sqref="F2:F1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=DropdownData!$A$1:$A$14</formula1>
-    </dataValidation>
-    <dataValidation sqref="G2:G1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=DropdownData!$B$1:$B$84</formula1>
-    </dataValidation>
+  <dataValidations count="1">
     <dataValidation sqref="H2:H1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=DropdownData!$C$1:$C$3</formula1>
     </dataValidation>

</xml_diff>

<commit_message>
changed as per the new req on june 11
</commit_message>
<xml_diff>
--- a/custom_import_template/static/xls/individual_import_template.xlsx
+++ b/custom_import_template/static/xls/individual_import_template.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -501,6 +501,16 @@
           <t>Status (Import)</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Disability Status</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -551,6 +561,16 @@
       <c r="J2" t="inlineStr">
         <is>
           <t>Active</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>0777123456</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>

</xml_diff>